<commit_message>
Se dinamizo la creacion del calendario
Se creo la funcion para que la creacion del calendario de cada mes sea dinamico.
</commit_message>
<xml_diff>
--- a/septiembre.xlsx
+++ b/septiembre.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/jhor_caro_virtualsoft_tech/Documents/Documentos/GitHub/Planeaci-n_SEO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="129" documentId="11_800C29F412E419F916FB06C293E467BE0930114B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF3E86EF-CA20-451A-A289-E7D25859078B}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="11_800C29F412E419F916FB06C293E467BE0930114B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4E77FE7-FB96-4B18-9966-468393EBCF28}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tareas de santiago septiembre" sheetId="1" r:id="rId1"/>
@@ -27,179 +27,28 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="5">
   <si>
     <t>Semana 1</t>
-  </si>
-  <si>
-    <t>01 Lunes / 5:45</t>
-  </si>
-  <si>
-    <t>02 Martes / 1:30</t>
-  </si>
-  <si>
-    <t>03 Miercoles / 5:00</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>04 Jueves /</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve"> 5:30</t>
-    </r>
-  </si>
-  <si>
-    <t>05 Viernes / 5:30</t>
   </si>
   <si>
     <t>Semana 2</t>
   </si>
   <si>
-    <t>08 Lunes / 3:30</t>
-  </si>
-  <si>
-    <t>9 Martes / 3:30</t>
-  </si>
-  <si>
-    <t>10 Miercoles / 3:45</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>11 Jueves /</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve"> 2:00</t>
-    </r>
-  </si>
-  <si>
-    <t>12 Viernes / 4:00</t>
-  </si>
-  <si>
     <t>Semana 3</t>
-  </si>
-  <si>
-    <t>15 Lunes / 2:30</t>
-  </si>
-  <si>
-    <t>16 Martes / 2:00</t>
-  </si>
-  <si>
-    <t>17 Miercoles / 2:00</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>18 Jueves /</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve"> 2:30</t>
-    </r>
-  </si>
-  <si>
-    <t>19 Viernes / 1:00</t>
   </si>
   <si>
     <t>Semana 4</t>
   </si>
   <si>
-    <t>22 Lunes / 1:45</t>
-  </si>
-  <si>
-    <t>23Martes / 4:30</t>
-  </si>
-  <si>
-    <t>24 Miercoles / 1:30</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>25 Jueves /</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve"> 6:00</t>
-    </r>
-  </si>
-  <si>
-    <t>26 Viernes / 5:30</t>
-  </si>
-  <si>
     <t>Semana 5</t>
-  </si>
-  <si>
-    <t>29 Lunes / 2:30</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve">30 viernes 12 /  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="22"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>1:45</t>
-    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -238,14 +87,8 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
-    <font>
-      <b/>
-      <sz val="22"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -274,12 +117,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEBF7FF"/>
         <bgColor rgb="FFEBF7FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFAE2D5"/>
-        <bgColor rgb="FFFAE2D5"/>
       </patternFill>
     </fill>
   </fills>
@@ -375,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -409,28 +246,19 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -439,6 +267,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -454,6 +288,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -675,30 +513,20 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:11" ht="28.5">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="C2" s="1"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="E2" s="1"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="3" t="s">
-        <v>3</v>
-      </c>
+      <c r="G2" s="3"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="I2" s="3"/>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="16"/>
+      <c r="A3" s="21"/>
       <c r="C3" s="4"/>
       <c r="E3" s="4"/>
       <c r="G3" s="4"/>
@@ -706,167 +534,167 @@
       <c r="K3" s="4"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="16"/>
+      <c r="A4" s="21"/>
       <c r="C4" s="5"/>
-      <c r="D4" s="18"/>
+      <c r="D4" s="17"/>
       <c r="E4" s="5"/>
-      <c r="F4" s="19"/>
+      <c r="F4" s="14"/>
       <c r="G4" s="5"/>
-      <c r="H4" s="19"/>
+      <c r="H4" s="14"/>
       <c r="I4" s="5"/>
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="16"/>
+      <c r="A5" s="21"/>
       <c r="C5" s="5"/>
-      <c r="D5" s="23"/>
+      <c r="D5" s="18"/>
       <c r="E5" s="5"/>
-      <c r="F5" s="21"/>
+      <c r="F5" s="15"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="21"/>
+      <c r="H5" s="15"/>
       <c r="I5" s="5"/>
       <c r="K5" s="5"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="16"/>
+      <c r="A6" s="21"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="23"/>
+      <c r="D6" s="18"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="21"/>
+      <c r="F6" s="15"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="21"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="5"/>
       <c r="K6" s="5"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="16"/>
+      <c r="A7" s="21"/>
       <c r="C7" s="5"/>
-      <c r="D7" s="23"/>
+      <c r="D7" s="18"/>
       <c r="E7" s="5"/>
-      <c r="F7" s="21"/>
+      <c r="F7" s="15"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="21"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="16"/>
+      <c r="A8" s="21"/>
       <c r="C8" s="5"/>
-      <c r="D8" s="23"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="5"/>
-      <c r="F8" s="21"/>
+      <c r="F8" s="15"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="21"/>
+      <c r="H8" s="15"/>
       <c r="I8" s="5"/>
       <c r="K8" s="5"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="20"/>
+      <c r="A9" s="22"/>
       <c r="C9" s="5"/>
-      <c r="D9" s="23"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="5"/>
-      <c r="F9" s="21"/>
+      <c r="F9" s="15"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="21"/>
+      <c r="H9" s="15"/>
       <c r="I9" s="5"/>
       <c r="K9" s="5"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="20"/>
+      <c r="A10" s="22"/>
       <c r="C10" s="5"/>
-      <c r="D10" s="23"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="21"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="21"/>
+      <c r="H10" s="15"/>
       <c r="I10" s="5"/>
       <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="20"/>
+      <c r="A11" s="22"/>
       <c r="C11" s="5"/>
-      <c r="D11" s="23"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="5"/>
-      <c r="F11" s="21"/>
+      <c r="F11" s="15"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="21"/>
+      <c r="H11" s="15"/>
       <c r="I11" s="5"/>
       <c r="K11" s="5"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="20"/>
+      <c r="A12" s="22"/>
       <c r="C12" s="5"/>
-      <c r="D12" s="23"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="5"/>
-      <c r="F12" s="21"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="21"/>
+      <c r="H12" s="15"/>
       <c r="I12" s="5"/>
       <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="20"/>
+      <c r="A13" s="22"/>
       <c r="C13" s="5"/>
-      <c r="D13" s="23"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="5"/>
-      <c r="F13" s="21"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="21"/>
+      <c r="H13" s="15"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="20"/>
+      <c r="A14" s="22"/>
       <c r="C14" s="5"/>
-      <c r="D14" s="23"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="5"/>
-      <c r="F14" s="21"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="21"/>
+      <c r="H14" s="15"/>
       <c r="I14" s="5"/>
       <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="16"/>
+      <c r="A15" s="21"/>
       <c r="C15" s="5"/>
-      <c r="D15" s="23"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="5"/>
-      <c r="F15" s="21"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="21"/>
+      <c r="H15" s="15"/>
       <c r="I15" s="5"/>
       <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="16"/>
+      <c r="A16" s="21"/>
       <c r="C16" s="5"/>
-      <c r="D16" s="23"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="5"/>
-      <c r="F16" s="21"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="6"/>
-      <c r="H16" s="21"/>
+      <c r="H16" s="15"/>
       <c r="I16" s="7"/>
       <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="16"/>
+      <c r="A17" s="21"/>
       <c r="C17" s="5"/>
-      <c r="D17" s="23"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="5"/>
-      <c r="F17" s="21"/>
+      <c r="F17" s="15"/>
       <c r="G17" s="6"/>
-      <c r="H17" s="21"/>
+      <c r="H17" s="15"/>
       <c r="I17" s="7"/>
       <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="17"/>
+      <c r="A18" s="23"/>
       <c r="C18" s="5"/>
-      <c r="D18" s="24"/>
+      <c r="D18" s="19"/>
       <c r="E18" s="5"/>
-      <c r="F18" s="22"/>
+      <c r="F18" s="16"/>
       <c r="G18" s="6"/>
-      <c r="H18" s="21"/>
+      <c r="H18" s="15"/>
       <c r="I18" s="7"/>
       <c r="K18" s="5"/>
     </row>
@@ -882,30 +710,20 @@
       <c r="K19" s="5"/>
     </row>
     <row r="21" spans="1:11" ht="28.5">
-      <c r="A21" s="15" t="s">
-        <v>6</v>
+      <c r="A21" s="20" t="s">
+        <v>1</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="C21" s="1"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="E21" s="1"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="G21" s="3"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="I21" s="3"/>
+      <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="16"/>
+      <c r="A22" s="21"/>
       <c r="C22" s="5"/>
       <c r="E22" s="5"/>
       <c r="G22" s="5"/>
@@ -913,7 +731,7 @@
       <c r="K22" s="5"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="20"/>
+      <c r="A23" s="22"/>
       <c r="C23" s="5"/>
       <c r="E23" s="5"/>
       <c r="G23" s="5"/>
@@ -921,7 +739,7 @@
       <c r="K23" s="5"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="20"/>
+      <c r="A24" s="22"/>
       <c r="C24" s="5"/>
       <c r="E24" s="5"/>
       <c r="G24" s="5"/>
@@ -929,7 +747,7 @@
       <c r="K24" s="5"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="20"/>
+      <c r="A25" s="22"/>
       <c r="C25" s="5"/>
       <c r="E25" s="5"/>
       <c r="G25" s="5"/>
@@ -937,7 +755,7 @@
       <c r="K25" s="5"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="20"/>
+      <c r="A26" s="22"/>
       <c r="C26" s="5"/>
       <c r="E26" s="5"/>
       <c r="G26" s="5"/>
@@ -945,7 +763,7 @@
       <c r="K26" s="5"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="20"/>
+      <c r="A27" s="22"/>
       <c r="C27" s="5"/>
       <c r="E27" s="5"/>
       <c r="G27" s="5"/>
@@ -953,7 +771,7 @@
       <c r="K27" s="5"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="20"/>
+      <c r="A28" s="22"/>
       <c r="C28" s="5"/>
       <c r="E28" s="5"/>
       <c r="G28" s="5"/>
@@ -961,7 +779,7 @@
       <c r="K28" s="5"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="16"/>
+      <c r="A29" s="21"/>
       <c r="C29" s="5"/>
       <c r="E29" s="5"/>
       <c r="G29" s="5"/>
@@ -969,7 +787,7 @@
       <c r="K29" s="5"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="16"/>
+      <c r="A30" s="21"/>
       <c r="C30" s="5"/>
       <c r="E30" s="5"/>
       <c r="G30" s="5"/>
@@ -977,7 +795,7 @@
       <c r="K30" s="5"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="16"/>
+      <c r="A31" s="21"/>
       <c r="C31" s="5"/>
       <c r="E31" s="5"/>
       <c r="G31" s="5"/>
@@ -985,7 +803,7 @@
       <c r="K31" s="5"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="16"/>
+      <c r="A32" s="21"/>
       <c r="C32" s="5"/>
       <c r="E32" s="5"/>
       <c r="G32" s="5"/>
@@ -993,7 +811,7 @@
       <c r="K32" s="5"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="16"/>
+      <c r="A33" s="21"/>
       <c r="C33" s="5"/>
       <c r="E33" s="5"/>
       <c r="G33" s="5"/>
@@ -1001,7 +819,7 @@
       <c r="K33" s="5"/>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="16"/>
+      <c r="A34" s="21"/>
       <c r="C34" s="7"/>
       <c r="E34" s="5"/>
       <c r="G34" s="5"/>
@@ -1009,7 +827,7 @@
       <c r="K34" s="7"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="17"/>
+      <c r="A35" s="23"/>
       <c r="C35" s="7"/>
       <c r="E35" s="5"/>
       <c r="G35" s="5"/>
@@ -1025,30 +843,20 @@
       <c r="K36" s="5"/>
     </row>
     <row r="38" spans="1:11" ht="28.5">
-      <c r="A38" s="15" t="s">
-        <v>12</v>
+      <c r="A38" s="20" t="s">
+        <v>2</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="C38" s="1"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E38" s="1"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="G38" s="3"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K38" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="I38" s="3"/>
+      <c r="K38" s="1"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="16"/>
+      <c r="A39" s="21"/>
       <c r="C39" s="5"/>
       <c r="D39" s="11"/>
       <c r="E39" s="5"/>
@@ -1057,7 +865,7 @@
       <c r="K39" s="5"/>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="16"/>
+      <c r="A40" s="21"/>
       <c r="C40" s="5"/>
       <c r="D40" s="12"/>
       <c r="E40" s="5"/>
@@ -1066,7 +874,7 @@
       <c r="K40" s="5"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="16"/>
+      <c r="A41" s="21"/>
       <c r="C41" s="5"/>
       <c r="D41" s="12"/>
       <c r="E41" s="5"/>
@@ -1075,7 +883,7 @@
       <c r="K41" s="5"/>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="16"/>
+      <c r="A42" s="21"/>
       <c r="C42" s="5"/>
       <c r="D42" s="12"/>
       <c r="E42" s="5"/>
@@ -1084,7 +892,7 @@
       <c r="K42" s="7"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="20"/>
+      <c r="A43" s="22"/>
       <c r="C43" s="5"/>
       <c r="D43" s="12"/>
       <c r="E43" s="5"/>
@@ -1093,7 +901,7 @@
       <c r="K43" s="7"/>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="20"/>
+      <c r="A44" s="22"/>
       <c r="C44" s="5"/>
       <c r="D44" s="12"/>
       <c r="E44" s="5"/>
@@ -1102,7 +910,7 @@
       <c r="K44" s="7"/>
     </row>
     <row r="45" spans="1:11">
-      <c r="A45" s="20"/>
+      <c r="A45" s="22"/>
       <c r="C45" s="5"/>
       <c r="D45" s="12"/>
       <c r="E45" s="5"/>
@@ -1111,7 +919,7 @@
       <c r="K45" s="7"/>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="20"/>
+      <c r="A46" s="22"/>
       <c r="C46" s="5"/>
       <c r="D46" s="12"/>
       <c r="E46" s="5"/>
@@ -1120,7 +928,7 @@
       <c r="K46" s="7"/>
     </row>
     <row r="47" spans="1:11">
-      <c r="A47" s="20"/>
+      <c r="A47" s="22"/>
       <c r="C47" s="5"/>
       <c r="D47" s="12"/>
       <c r="E47" s="5"/>
@@ -1129,7 +937,7 @@
       <c r="K47" s="7"/>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="20"/>
+      <c r="A48" s="22"/>
       <c r="C48" s="5"/>
       <c r="D48" s="12"/>
       <c r="E48" s="5"/>
@@ -1138,7 +946,7 @@
       <c r="K48" s="7"/>
     </row>
     <row r="49" spans="1:11">
-      <c r="A49" s="20"/>
+      <c r="A49" s="22"/>
       <c r="C49" s="5"/>
       <c r="D49" s="12"/>
       <c r="E49" s="5"/>
@@ -1147,7 +955,7 @@
       <c r="K49" s="7"/>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="20"/>
+      <c r="A50" s="22"/>
       <c r="C50" s="5"/>
       <c r="D50" s="12"/>
       <c r="E50" s="5"/>
@@ -1156,7 +964,7 @@
       <c r="K50" s="7"/>
     </row>
     <row r="51" spans="1:11">
-      <c r="A51" s="16"/>
+      <c r="A51" s="21"/>
       <c r="C51" s="5"/>
       <c r="D51" s="12"/>
       <c r="E51" s="5"/>
@@ -1165,7 +973,7 @@
       <c r="K51" s="7"/>
     </row>
     <row r="52" spans="1:11">
-      <c r="A52" s="16"/>
+      <c r="A52" s="21"/>
       <c r="C52" s="5"/>
       <c r="D52" s="12"/>
       <c r="E52" s="5"/>
@@ -1174,7 +982,7 @@
       <c r="K52" s="7"/>
     </row>
     <row r="53" spans="1:11">
-      <c r="A53" s="17"/>
+      <c r="A53" s="23"/>
       <c r="C53" s="5"/>
       <c r="D53" s="12"/>
       <c r="E53" s="5"/>
@@ -1183,30 +991,20 @@
       <c r="K53" s="7"/>
     </row>
     <row r="55" spans="1:11" ht="28.5">
-      <c r="A55" s="15" t="s">
-        <v>18</v>
+      <c r="A55" s="20" t="s">
+        <v>3</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="C55" s="1"/>
       <c r="D55" s="2"/>
-      <c r="E55" s="1" t="s">
-        <v>20</v>
-      </c>
+      <c r="E55" s="1"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="G55" s="3"/>
       <c r="H55" s="2"/>
-      <c r="I55" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="I55" s="3"/>
+      <c r="K55" s="1"/>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="16"/>
+      <c r="A56" s="21"/>
       <c r="C56" s="5"/>
       <c r="E56" s="5"/>
       <c r="G56" s="5"/>
@@ -1214,7 +1012,7 @@
       <c r="K56" s="5"/>
     </row>
     <row r="57" spans="1:11">
-      <c r="A57" s="16"/>
+      <c r="A57" s="21"/>
       <c r="C57" s="5"/>
       <c r="E57" s="5"/>
       <c r="G57" s="5"/>
@@ -1222,7 +1020,7 @@
       <c r="K57" s="5"/>
     </row>
     <row r="58" spans="1:11">
-      <c r="A58" s="16"/>
+      <c r="A58" s="21"/>
       <c r="C58" s="5"/>
       <c r="E58" s="5"/>
       <c r="G58" s="5"/>
@@ -1230,7 +1028,7 @@
       <c r="K58" s="5"/>
     </row>
     <row r="59" spans="1:11">
-      <c r="A59" s="16"/>
+      <c r="A59" s="21"/>
       <c r="C59" s="5"/>
       <c r="E59" s="5"/>
       <c r="G59" s="5"/>
@@ -1238,7 +1036,7 @@
       <c r="K59" s="5"/>
     </row>
     <row r="60" spans="1:11">
-      <c r="A60" s="20"/>
+      <c r="A60" s="22"/>
       <c r="C60" s="5"/>
       <c r="E60" s="5"/>
       <c r="G60" s="5"/>
@@ -1246,7 +1044,7 @@
       <c r="K60" s="5"/>
     </row>
     <row r="61" spans="1:11">
-      <c r="A61" s="20"/>
+      <c r="A61" s="22"/>
       <c r="C61" s="5"/>
       <c r="E61" s="5"/>
       <c r="G61" s="5"/>
@@ -1254,7 +1052,7 @@
       <c r="K61" s="5"/>
     </row>
     <row r="62" spans="1:11">
-      <c r="A62" s="20"/>
+      <c r="A62" s="22"/>
       <c r="C62" s="5"/>
       <c r="E62" s="5"/>
       <c r="G62" s="5"/>
@@ -1262,7 +1060,7 @@
       <c r="K62" s="5"/>
     </row>
     <row r="63" spans="1:11">
-      <c r="A63" s="20"/>
+      <c r="A63" s="22"/>
       <c r="C63" s="5"/>
       <c r="E63" s="5"/>
       <c r="G63" s="5"/>
@@ -1270,7 +1068,7 @@
       <c r="K63" s="5"/>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" s="20"/>
+      <c r="A64" s="22"/>
       <c r="C64" s="5"/>
       <c r="E64" s="5"/>
       <c r="G64" s="5"/>
@@ -1278,7 +1076,7 @@
       <c r="K64" s="5"/>
     </row>
     <row r="65" spans="1:11">
-      <c r="A65" s="20"/>
+      <c r="A65" s="22"/>
       <c r="C65" s="5"/>
       <c r="E65" s="5"/>
       <c r="G65" s="5"/>
@@ -1286,7 +1084,7 @@
       <c r="K65" s="5"/>
     </row>
     <row r="66" spans="1:11">
-      <c r="A66" s="16"/>
+      <c r="A66" s="21"/>
       <c r="C66" s="5"/>
       <c r="E66" s="5"/>
       <c r="G66" s="5"/>
@@ -1294,7 +1092,7 @@
       <c r="K66" s="5"/>
     </row>
     <row r="67" spans="1:11">
-      <c r="A67" s="16"/>
+      <c r="A67" s="21"/>
       <c r="C67" s="7"/>
       <c r="E67" s="5"/>
       <c r="G67" s="5"/>
@@ -1302,7 +1100,7 @@
       <c r="K67" s="5"/>
     </row>
     <row r="68" spans="1:11">
-      <c r="A68" s="16"/>
+      <c r="A68" s="21"/>
       <c r="C68" s="7"/>
       <c r="E68" s="5"/>
       <c r="G68" s="5"/>
@@ -1310,7 +1108,7 @@
       <c r="K68" s="5"/>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="16"/>
+      <c r="A69" s="21"/>
       <c r="C69" s="7"/>
       <c r="E69" s="5"/>
       <c r="G69" s="5"/>
@@ -1318,7 +1116,7 @@
       <c r="K69" s="5"/>
     </row>
     <row r="70" spans="1:11">
-      <c r="A70" s="17"/>
+      <c r="A70" s="23"/>
       <c r="C70" s="7"/>
       <c r="E70" s="5"/>
       <c r="G70" s="7"/>
@@ -1326,93 +1124,89 @@
       <c r="K70" s="5"/>
     </row>
     <row r="72" spans="1:11" ht="28.5">
-      <c r="A72" s="15" t="s">
-        <v>24</v>
+      <c r="A72" s="20" t="s">
+        <v>4</v>
       </c>
-      <c r="C72" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="C72" s="1"/>
+      <c r="E72" s="3"/>
     </row>
     <row r="73" spans="1:11">
-      <c r="A73" s="16"/>
+      <c r="A73" s="21"/>
       <c r="C73" s="4"/>
-      <c r="E73" s="14"/>
+      <c r="E73" s="13"/>
     </row>
     <row r="74" spans="1:11">
-      <c r="A74" s="16"/>
+      <c r="A74" s="21"/>
       <c r="C74" s="5"/>
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="1:11">
-      <c r="A75" s="16"/>
+      <c r="A75" s="21"/>
       <c r="C75" s="5"/>
       <c r="E75" s="5"/>
     </row>
     <row r="76" spans="1:11">
-      <c r="A76" s="20"/>
+      <c r="A76" s="22"/>
       <c r="C76" s="5"/>
       <c r="E76" s="5"/>
     </row>
     <row r="77" spans="1:11">
-      <c r="A77" s="20"/>
+      <c r="A77" s="22"/>
       <c r="C77" s="5"/>
       <c r="E77" s="5"/>
     </row>
     <row r="78" spans="1:11">
-      <c r="A78" s="20"/>
+      <c r="A78" s="22"/>
       <c r="C78" s="5"/>
       <c r="E78" s="5"/>
     </row>
     <row r="79" spans="1:11">
-      <c r="A79" s="20"/>
+      <c r="A79" s="22"/>
       <c r="C79" s="5"/>
       <c r="E79" s="5"/>
     </row>
     <row r="80" spans="1:11">
-      <c r="A80" s="20"/>
+      <c r="A80" s="22"/>
       <c r="C80" s="5"/>
       <c r="E80" s="5"/>
     </row>
     <row r="81" spans="1:5">
-      <c r="A81" s="20"/>
+      <c r="A81" s="22"/>
       <c r="C81" s="5"/>
       <c r="E81" s="5"/>
     </row>
     <row r="82" spans="1:5">
-      <c r="A82" s="20"/>
+      <c r="A82" s="22"/>
       <c r="C82" s="5"/>
       <c r="E82" s="5"/>
     </row>
     <row r="83" spans="1:5">
-      <c r="A83" s="20"/>
+      <c r="A83" s="22"/>
       <c r="C83" s="5"/>
       <c r="E83" s="5"/>
     </row>
     <row r="84" spans="1:5">
-      <c r="A84" s="16"/>
+      <c r="A84" s="21"/>
       <c r="C84" s="5"/>
       <c r="E84" s="5"/>
     </row>
     <row r="85" spans="1:5">
-      <c r="A85" s="20"/>
+      <c r="A85" s="22"/>
       <c r="C85" s="5"/>
       <c r="E85" s="5"/>
     </row>
     <row r="86" spans="1:5">
-      <c r="A86" s="20"/>
+      <c r="A86" s="22"/>
       <c r="C86" s="5"/>
       <c r="E86" s="5"/>
     </row>
     <row r="87" spans="1:5">
-      <c r="A87" s="16"/>
+      <c r="A87" s="21"/>
       <c r="C87" s="5"/>
       <c r="E87" s="5"/>
     </row>
     <row r="88" spans="1:5">
-      <c r="A88" s="17"/>
+      <c r="A88" s="23"/>
       <c r="C88" s="5"/>
       <c r="E88" s="5"/>
     </row>
@@ -1455,30 +1249,20 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:11" ht="28.5">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="C2" s="1"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="E2" s="1"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="3" t="s">
-        <v>3</v>
-      </c>
+      <c r="G2" s="3"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="I2" s="3"/>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="16"/>
+      <c r="A3" s="21"/>
       <c r="C3" s="4"/>
       <c r="E3" s="4"/>
       <c r="G3" s="4"/>
@@ -1486,167 +1270,167 @@
       <c r="K3" s="4"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="16"/>
+      <c r="A4" s="21"/>
       <c r="C4" s="5"/>
-      <c r="D4" s="18"/>
+      <c r="D4" s="17"/>
       <c r="E4" s="5"/>
-      <c r="F4" s="19"/>
+      <c r="F4" s="14"/>
       <c r="G4" s="5"/>
-      <c r="H4" s="19"/>
+      <c r="H4" s="14"/>
       <c r="I4" s="5"/>
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="16"/>
+      <c r="A5" s="21"/>
       <c r="C5" s="5"/>
-      <c r="D5" s="23"/>
+      <c r="D5" s="18"/>
       <c r="E5" s="5"/>
-      <c r="F5" s="21"/>
+      <c r="F5" s="15"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="21"/>
+      <c r="H5" s="15"/>
       <c r="I5" s="5"/>
       <c r="K5" s="5"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="16"/>
+      <c r="A6" s="21"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="23"/>
+      <c r="D6" s="18"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="21"/>
+      <c r="F6" s="15"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="21"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="5"/>
       <c r="K6" s="5"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="16"/>
+      <c r="A7" s="21"/>
       <c r="C7" s="5"/>
-      <c r="D7" s="23"/>
+      <c r="D7" s="18"/>
       <c r="E7" s="5"/>
-      <c r="F7" s="21"/>
+      <c r="F7" s="15"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="21"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="16"/>
+      <c r="A8" s="21"/>
       <c r="C8" s="5"/>
-      <c r="D8" s="23"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="5"/>
-      <c r="F8" s="21"/>
+      <c r="F8" s="15"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="21"/>
+      <c r="H8" s="15"/>
       <c r="I8" s="5"/>
       <c r="K8" s="5"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="20"/>
+      <c r="A9" s="22"/>
       <c r="C9" s="5"/>
-      <c r="D9" s="23"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="5"/>
-      <c r="F9" s="21"/>
+      <c r="F9" s="15"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="21"/>
+      <c r="H9" s="15"/>
       <c r="I9" s="5"/>
       <c r="K9" s="5"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="20"/>
+      <c r="A10" s="22"/>
       <c r="C10" s="5"/>
-      <c r="D10" s="23"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="21"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="21"/>
+      <c r="H10" s="15"/>
       <c r="I10" s="5"/>
       <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="20"/>
+      <c r="A11" s="22"/>
       <c r="C11" s="5"/>
-      <c r="D11" s="23"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="5"/>
-      <c r="F11" s="21"/>
+      <c r="F11" s="15"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="21"/>
+      <c r="H11" s="15"/>
       <c r="I11" s="5"/>
       <c r="K11" s="5"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="20"/>
+      <c r="A12" s="22"/>
       <c r="C12" s="5"/>
-      <c r="D12" s="23"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="5"/>
-      <c r="F12" s="21"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="21"/>
+      <c r="H12" s="15"/>
       <c r="I12" s="5"/>
       <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="20"/>
+      <c r="A13" s="22"/>
       <c r="C13" s="5"/>
-      <c r="D13" s="23"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="5"/>
-      <c r="F13" s="21"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="21"/>
+      <c r="H13" s="15"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="20"/>
+      <c r="A14" s="22"/>
       <c r="C14" s="5"/>
-      <c r="D14" s="23"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="5"/>
-      <c r="F14" s="21"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="21"/>
+      <c r="H14" s="15"/>
       <c r="I14" s="5"/>
       <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="16"/>
+      <c r="A15" s="21"/>
       <c r="C15" s="5"/>
-      <c r="D15" s="23"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="5"/>
-      <c r="F15" s="21"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="21"/>
+      <c r="H15" s="15"/>
       <c r="I15" s="5"/>
       <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="16"/>
+      <c r="A16" s="21"/>
       <c r="C16" s="5"/>
-      <c r="D16" s="23"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="5"/>
-      <c r="F16" s="21"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="6"/>
-      <c r="H16" s="21"/>
+      <c r="H16" s="15"/>
       <c r="I16" s="7"/>
       <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="16"/>
+      <c r="A17" s="21"/>
       <c r="C17" s="5"/>
-      <c r="D17" s="23"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="5"/>
-      <c r="F17" s="21"/>
+      <c r="F17" s="15"/>
       <c r="G17" s="6"/>
-      <c r="H17" s="21"/>
+      <c r="H17" s="15"/>
       <c r="I17" s="7"/>
       <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="17"/>
+      <c r="A18" s="23"/>
       <c r="C18" s="5"/>
-      <c r="D18" s="24"/>
+      <c r="D18" s="19"/>
       <c r="E18" s="5"/>
-      <c r="F18" s="22"/>
+      <c r="F18" s="16"/>
       <c r="G18" s="6"/>
-      <c r="H18" s="21"/>
+      <c r="H18" s="15"/>
       <c r="I18" s="7"/>
       <c r="K18" s="5"/>
     </row>
@@ -1662,30 +1446,20 @@
       <c r="K19" s="5"/>
     </row>
     <row r="21" spans="1:11" ht="28.5">
-      <c r="A21" s="15" t="s">
-        <v>6</v>
+      <c r="A21" s="20" t="s">
+        <v>1</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="C21" s="1"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="E21" s="1"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="G21" s="3"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="I21" s="3"/>
+      <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="16"/>
+      <c r="A22" s="21"/>
       <c r="C22" s="5"/>
       <c r="E22" s="5"/>
       <c r="G22" s="5"/>
@@ -1693,7 +1467,7 @@
       <c r="K22" s="5"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="20"/>
+      <c r="A23" s="22"/>
       <c r="C23" s="5"/>
       <c r="E23" s="5"/>
       <c r="G23" s="5"/>
@@ -1701,7 +1475,7 @@
       <c r="K23" s="5"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="20"/>
+      <c r="A24" s="22"/>
       <c r="C24" s="5"/>
       <c r="E24" s="5"/>
       <c r="G24" s="5"/>
@@ -1709,7 +1483,7 @@
       <c r="K24" s="5"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="20"/>
+      <c r="A25" s="22"/>
       <c r="C25" s="5"/>
       <c r="E25" s="5"/>
       <c r="G25" s="5"/>
@@ -1717,7 +1491,7 @@
       <c r="K25" s="5"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="20"/>
+      <c r="A26" s="22"/>
       <c r="C26" s="5"/>
       <c r="E26" s="5"/>
       <c r="G26" s="5"/>
@@ -1725,7 +1499,7 @@
       <c r="K26" s="5"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="20"/>
+      <c r="A27" s="22"/>
       <c r="C27" s="5"/>
       <c r="E27" s="5"/>
       <c r="G27" s="5"/>
@@ -1733,7 +1507,7 @@
       <c r="K27" s="5"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="20"/>
+      <c r="A28" s="22"/>
       <c r="C28" s="5"/>
       <c r="E28" s="5"/>
       <c r="G28" s="5"/>
@@ -1741,7 +1515,7 @@
       <c r="K28" s="5"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="16"/>
+      <c r="A29" s="21"/>
       <c r="C29" s="5"/>
       <c r="E29" s="5"/>
       <c r="G29" s="5"/>
@@ -1749,7 +1523,7 @@
       <c r="K29" s="5"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="16"/>
+      <c r="A30" s="21"/>
       <c r="C30" s="5"/>
       <c r="E30" s="5"/>
       <c r="G30" s="5"/>
@@ -1757,7 +1531,7 @@
       <c r="K30" s="5"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="16"/>
+      <c r="A31" s="21"/>
       <c r="C31" s="5"/>
       <c r="E31" s="5"/>
       <c r="G31" s="5"/>
@@ -1765,7 +1539,7 @@
       <c r="K31" s="5"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="16"/>
+      <c r="A32" s="21"/>
       <c r="C32" s="5"/>
       <c r="E32" s="5"/>
       <c r="G32" s="5"/>
@@ -1773,7 +1547,7 @@
       <c r="K32" s="5"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="16"/>
+      <c r="A33" s="21"/>
       <c r="C33" s="5"/>
       <c r="E33" s="5"/>
       <c r="G33" s="5"/>
@@ -1781,7 +1555,7 @@
       <c r="K33" s="5"/>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="16"/>
+      <c r="A34" s="21"/>
       <c r="C34" s="7"/>
       <c r="E34" s="5"/>
       <c r="G34" s="5"/>
@@ -1789,7 +1563,7 @@
       <c r="K34" s="7"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="17"/>
+      <c r="A35" s="23"/>
       <c r="C35" s="7"/>
       <c r="E35" s="5"/>
       <c r="G35" s="5"/>
@@ -1805,30 +1579,20 @@
       <c r="K36" s="5"/>
     </row>
     <row r="38" spans="1:11" ht="28.5">
-      <c r="A38" s="15" t="s">
-        <v>12</v>
+      <c r="A38" s="20" t="s">
+        <v>2</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="C38" s="1"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E38" s="1"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="G38" s="3"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K38" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="I38" s="3"/>
+      <c r="K38" s="1"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="16"/>
+      <c r="A39" s="21"/>
       <c r="C39" s="5"/>
       <c r="D39" s="11"/>
       <c r="E39" s="5"/>
@@ -1837,7 +1601,7 @@
       <c r="K39" s="5"/>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="16"/>
+      <c r="A40" s="21"/>
       <c r="C40" s="5"/>
       <c r="D40" s="12"/>
       <c r="E40" s="5"/>
@@ -1846,7 +1610,7 @@
       <c r="K40" s="5"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="16"/>
+      <c r="A41" s="21"/>
       <c r="C41" s="5"/>
       <c r="D41" s="12"/>
       <c r="E41" s="5"/>
@@ -1855,7 +1619,7 @@
       <c r="K41" s="5"/>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="16"/>
+      <c r="A42" s="21"/>
       <c r="C42" s="5"/>
       <c r="D42" s="12"/>
       <c r="E42" s="5"/>
@@ -1864,7 +1628,7 @@
       <c r="K42" s="7"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="20"/>
+      <c r="A43" s="22"/>
       <c r="C43" s="5"/>
       <c r="D43" s="12"/>
       <c r="E43" s="5"/>
@@ -1873,7 +1637,7 @@
       <c r="K43" s="7"/>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="20"/>
+      <c r="A44" s="22"/>
       <c r="C44" s="5"/>
       <c r="D44" s="12"/>
       <c r="E44" s="5"/>
@@ -1882,7 +1646,7 @@
       <c r="K44" s="7"/>
     </row>
     <row r="45" spans="1:11">
-      <c r="A45" s="20"/>
+      <c r="A45" s="22"/>
       <c r="C45" s="5"/>
       <c r="D45" s="12"/>
       <c r="E45" s="5"/>
@@ -1891,7 +1655,7 @@
       <c r="K45" s="7"/>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="20"/>
+      <c r="A46" s="22"/>
       <c r="C46" s="5"/>
       <c r="D46" s="12"/>
       <c r="E46" s="5"/>
@@ -1900,7 +1664,7 @@
       <c r="K46" s="7"/>
     </row>
     <row r="47" spans="1:11">
-      <c r="A47" s="20"/>
+      <c r="A47" s="22"/>
       <c r="C47" s="5"/>
       <c r="D47" s="12"/>
       <c r="E47" s="5"/>
@@ -1909,7 +1673,7 @@
       <c r="K47" s="7"/>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="20"/>
+      <c r="A48" s="22"/>
       <c r="C48" s="5"/>
       <c r="D48" s="12"/>
       <c r="E48" s="5"/>
@@ -1918,7 +1682,7 @@
       <c r="K48" s="7"/>
     </row>
     <row r="49" spans="1:11">
-      <c r="A49" s="20"/>
+      <c r="A49" s="22"/>
       <c r="C49" s="5"/>
       <c r="D49" s="12"/>
       <c r="E49" s="5"/>
@@ -1927,7 +1691,7 @@
       <c r="K49" s="7"/>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="20"/>
+      <c r="A50" s="22"/>
       <c r="C50" s="5"/>
       <c r="D50" s="12"/>
       <c r="E50" s="5"/>
@@ -1936,7 +1700,7 @@
       <c r="K50" s="7"/>
     </row>
     <row r="51" spans="1:11">
-      <c r="A51" s="16"/>
+      <c r="A51" s="21"/>
       <c r="C51" s="5"/>
       <c r="D51" s="12"/>
       <c r="E51" s="5"/>
@@ -1945,7 +1709,7 @@
       <c r="K51" s="7"/>
     </row>
     <row r="52" spans="1:11">
-      <c r="A52" s="16"/>
+      <c r="A52" s="21"/>
       <c r="C52" s="5"/>
       <c r="D52" s="12"/>
       <c r="E52" s="5"/>
@@ -1954,7 +1718,7 @@
       <c r="K52" s="7"/>
     </row>
     <row r="53" spans="1:11">
-      <c r="A53" s="17"/>
+      <c r="A53" s="23"/>
       <c r="C53" s="5"/>
       <c r="D53" s="12"/>
       <c r="E53" s="5"/>
@@ -1963,30 +1727,20 @@
       <c r="K53" s="7"/>
     </row>
     <row r="55" spans="1:11" ht="28.5">
-      <c r="A55" s="15" t="s">
-        <v>18</v>
+      <c r="A55" s="20" t="s">
+        <v>3</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="C55" s="1"/>
       <c r="D55" s="2"/>
-      <c r="E55" s="1" t="s">
-        <v>20</v>
-      </c>
+      <c r="E55" s="1"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="G55" s="3"/>
       <c r="H55" s="2"/>
-      <c r="I55" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="I55" s="3"/>
+      <c r="K55" s="1"/>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="16"/>
+      <c r="A56" s="21"/>
       <c r="C56" s="5"/>
       <c r="E56" s="5"/>
       <c r="G56" s="5"/>
@@ -1994,7 +1748,7 @@
       <c r="K56" s="5"/>
     </row>
     <row r="57" spans="1:11">
-      <c r="A57" s="16"/>
+      <c r="A57" s="21"/>
       <c r="C57" s="5"/>
       <c r="E57" s="5"/>
       <c r="G57" s="5"/>
@@ -2002,7 +1756,7 @@
       <c r="K57" s="5"/>
     </row>
     <row r="58" spans="1:11">
-      <c r="A58" s="16"/>
+      <c r="A58" s="21"/>
       <c r="C58" s="5"/>
       <c r="E58" s="5"/>
       <c r="G58" s="5"/>
@@ -2010,7 +1764,7 @@
       <c r="K58" s="5"/>
     </row>
     <row r="59" spans="1:11">
-      <c r="A59" s="16"/>
+      <c r="A59" s="21"/>
       <c r="C59" s="5"/>
       <c r="E59" s="5"/>
       <c r="G59" s="5"/>
@@ -2018,7 +1772,7 @@
       <c r="K59" s="5"/>
     </row>
     <row r="60" spans="1:11">
-      <c r="A60" s="20"/>
+      <c r="A60" s="22"/>
       <c r="C60" s="5"/>
       <c r="E60" s="5"/>
       <c r="G60" s="5"/>
@@ -2026,7 +1780,7 @@
       <c r="K60" s="5"/>
     </row>
     <row r="61" spans="1:11">
-      <c r="A61" s="20"/>
+      <c r="A61" s="22"/>
       <c r="C61" s="5"/>
       <c r="E61" s="5"/>
       <c r="G61" s="5"/>
@@ -2034,7 +1788,7 @@
       <c r="K61" s="5"/>
     </row>
     <row r="62" spans="1:11">
-      <c r="A62" s="20"/>
+      <c r="A62" s="22"/>
       <c r="C62" s="5"/>
       <c r="E62" s="5"/>
       <c r="G62" s="5"/>
@@ -2042,7 +1796,7 @@
       <c r="K62" s="5"/>
     </row>
     <row r="63" spans="1:11">
-      <c r="A63" s="20"/>
+      <c r="A63" s="22"/>
       <c r="C63" s="5"/>
       <c r="E63" s="5"/>
       <c r="G63" s="5"/>
@@ -2050,7 +1804,7 @@
       <c r="K63" s="5"/>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" s="20"/>
+      <c r="A64" s="22"/>
       <c r="C64" s="5"/>
       <c r="E64" s="5"/>
       <c r="G64" s="5"/>
@@ -2058,7 +1812,7 @@
       <c r="K64" s="5"/>
     </row>
     <row r="65" spans="1:11">
-      <c r="A65" s="20"/>
+      <c r="A65" s="22"/>
       <c r="C65" s="5"/>
       <c r="E65" s="5"/>
       <c r="G65" s="5"/>
@@ -2066,7 +1820,7 @@
       <c r="K65" s="5"/>
     </row>
     <row r="66" spans="1:11">
-      <c r="A66" s="16"/>
+      <c r="A66" s="21"/>
       <c r="C66" s="5"/>
       <c r="E66" s="5"/>
       <c r="G66" s="5"/>
@@ -2074,7 +1828,7 @@
       <c r="K66" s="5"/>
     </row>
     <row r="67" spans="1:11">
-      <c r="A67" s="16"/>
+      <c r="A67" s="21"/>
       <c r="C67" s="7"/>
       <c r="E67" s="5"/>
       <c r="G67" s="5"/>
@@ -2082,7 +1836,7 @@
       <c r="K67" s="5"/>
     </row>
     <row r="68" spans="1:11">
-      <c r="A68" s="16"/>
+      <c r="A68" s="21"/>
       <c r="C68" s="7"/>
       <c r="E68" s="5"/>
       <c r="G68" s="5"/>
@@ -2090,7 +1844,7 @@
       <c r="K68" s="5"/>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="16"/>
+      <c r="A69" s="21"/>
       <c r="C69" s="7"/>
       <c r="E69" s="5"/>
       <c r="G69" s="5"/>
@@ -2098,7 +1852,7 @@
       <c r="K69" s="5"/>
     </row>
     <row r="70" spans="1:11">
-      <c r="A70" s="17"/>
+      <c r="A70" s="23"/>
       <c r="C70" s="7"/>
       <c r="E70" s="5"/>
       <c r="G70" s="7"/>
@@ -2106,93 +1860,89 @@
       <c r="K70" s="5"/>
     </row>
     <row r="72" spans="1:11" ht="28.5">
-      <c r="A72" s="15" t="s">
-        <v>24</v>
+      <c r="A72" s="20" t="s">
+        <v>4</v>
       </c>
-      <c r="C72" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="C72" s="1"/>
+      <c r="E72" s="3"/>
     </row>
     <row r="73" spans="1:11">
-      <c r="A73" s="16"/>
+      <c r="A73" s="21"/>
       <c r="C73" s="4"/>
-      <c r="E73" s="14"/>
+      <c r="E73" s="13"/>
     </row>
     <row r="74" spans="1:11">
-      <c r="A74" s="16"/>
+      <c r="A74" s="21"/>
       <c r="C74" s="5"/>
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="1:11">
-      <c r="A75" s="16"/>
+      <c r="A75" s="21"/>
       <c r="C75" s="5"/>
       <c r="E75" s="5"/>
     </row>
     <row r="76" spans="1:11">
-      <c r="A76" s="20"/>
+      <c r="A76" s="22"/>
       <c r="C76" s="5"/>
       <c r="E76" s="5"/>
     </row>
     <row r="77" spans="1:11">
-      <c r="A77" s="20"/>
+      <c r="A77" s="22"/>
       <c r="C77" s="5"/>
       <c r="E77" s="5"/>
     </row>
     <row r="78" spans="1:11">
-      <c r="A78" s="20"/>
+      <c r="A78" s="22"/>
       <c r="C78" s="5"/>
       <c r="E78" s="5"/>
     </row>
     <row r="79" spans="1:11">
-      <c r="A79" s="20"/>
+      <c r="A79" s="22"/>
       <c r="C79" s="5"/>
       <c r="E79" s="5"/>
     </row>
     <row r="80" spans="1:11">
-      <c r="A80" s="20"/>
+      <c r="A80" s="22"/>
       <c r="C80" s="5"/>
       <c r="E80" s="5"/>
     </row>
     <row r="81" spans="1:5">
-      <c r="A81" s="20"/>
+      <c r="A81" s="22"/>
       <c r="C81" s="5"/>
       <c r="E81" s="5"/>
     </row>
     <row r="82" spans="1:5">
-      <c r="A82" s="20"/>
+      <c r="A82" s="22"/>
       <c r="C82" s="5"/>
       <c r="E82" s="5"/>
     </row>
     <row r="83" spans="1:5">
-      <c r="A83" s="20"/>
+      <c r="A83" s="22"/>
       <c r="C83" s="5"/>
       <c r="E83" s="5"/>
     </row>
     <row r="84" spans="1:5">
-      <c r="A84" s="16"/>
+      <c r="A84" s="21"/>
       <c r="C84" s="5"/>
       <c r="E84" s="5"/>
     </row>
     <row r="85" spans="1:5">
-      <c r="A85" s="20"/>
+      <c r="A85" s="22"/>
       <c r="C85" s="5"/>
       <c r="E85" s="5"/>
     </row>
     <row r="86" spans="1:5">
-      <c r="A86" s="20"/>
+      <c r="A86" s="22"/>
       <c r="C86" s="5"/>
       <c r="E86" s="5"/>
     </row>
     <row r="87" spans="1:5">
-      <c r="A87" s="16"/>
+      <c r="A87" s="21"/>
       <c r="C87" s="5"/>
       <c r="E87" s="5"/>
     </row>
     <row r="88" spans="1:5">
-      <c r="A88" s="17"/>
+      <c r="A88" s="23"/>
       <c r="C88" s="5"/>
       <c r="E88" s="5"/>
     </row>
@@ -2235,30 +1985,20 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:11" ht="28.5">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="C2" s="1"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="E2" s="1"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="3" t="s">
-        <v>3</v>
-      </c>
+      <c r="G2" s="3"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="I2" s="3"/>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="16"/>
+      <c r="A3" s="21"/>
       <c r="C3" s="4"/>
       <c r="E3" s="4"/>
       <c r="G3" s="4"/>
@@ -2266,167 +2006,167 @@
       <c r="K3" s="4"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="16"/>
+      <c r="A4" s="21"/>
       <c r="C4" s="5"/>
-      <c r="D4" s="18"/>
+      <c r="D4" s="17"/>
       <c r="E4" s="5"/>
-      <c r="F4" s="19"/>
+      <c r="F4" s="14"/>
       <c r="G4" s="5"/>
-      <c r="H4" s="19"/>
+      <c r="H4" s="14"/>
       <c r="I4" s="5"/>
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="16"/>
+      <c r="A5" s="21"/>
       <c r="C5" s="5"/>
-      <c r="D5" s="23"/>
+      <c r="D5" s="18"/>
       <c r="E5" s="5"/>
-      <c r="F5" s="21"/>
+      <c r="F5" s="15"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="21"/>
+      <c r="H5" s="15"/>
       <c r="I5" s="5"/>
       <c r="K5" s="5"/>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="16"/>
+      <c r="A6" s="21"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="23"/>
+      <c r="D6" s="18"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="21"/>
+      <c r="F6" s="15"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="21"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="5"/>
       <c r="K6" s="5"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="16"/>
+      <c r="A7" s="21"/>
       <c r="C7" s="5"/>
-      <c r="D7" s="23"/>
+      <c r="D7" s="18"/>
       <c r="E7" s="5"/>
-      <c r="F7" s="21"/>
+      <c r="F7" s="15"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="21"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="5"/>
       <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="16"/>
+      <c r="A8" s="21"/>
       <c r="C8" s="5"/>
-      <c r="D8" s="23"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="5"/>
-      <c r="F8" s="21"/>
+      <c r="F8" s="15"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="21"/>
+      <c r="H8" s="15"/>
       <c r="I8" s="5"/>
       <c r="K8" s="5"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="20"/>
+      <c r="A9" s="22"/>
       <c r="C9" s="5"/>
-      <c r="D9" s="23"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="5"/>
-      <c r="F9" s="21"/>
+      <c r="F9" s="15"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="21"/>
+      <c r="H9" s="15"/>
       <c r="I9" s="5"/>
       <c r="K9" s="5"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="20"/>
+      <c r="A10" s="22"/>
       <c r="C10" s="5"/>
-      <c r="D10" s="23"/>
+      <c r="D10" s="18"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="21"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="21"/>
+      <c r="H10" s="15"/>
       <c r="I10" s="5"/>
       <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="20"/>
+      <c r="A11" s="22"/>
       <c r="C11" s="5"/>
-      <c r="D11" s="23"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="5"/>
-      <c r="F11" s="21"/>
+      <c r="F11" s="15"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="21"/>
+      <c r="H11" s="15"/>
       <c r="I11" s="5"/>
       <c r="K11" s="5"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="20"/>
+      <c r="A12" s="22"/>
       <c r="C12" s="5"/>
-      <c r="D12" s="23"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="5"/>
-      <c r="F12" s="21"/>
+      <c r="F12" s="15"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="21"/>
+      <c r="H12" s="15"/>
       <c r="I12" s="5"/>
       <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="20"/>
+      <c r="A13" s="22"/>
       <c r="C13" s="5"/>
-      <c r="D13" s="23"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="5"/>
-      <c r="F13" s="21"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="21"/>
+      <c r="H13" s="15"/>
       <c r="I13" s="5"/>
       <c r="K13" s="5"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="20"/>
+      <c r="A14" s="22"/>
       <c r="C14" s="5"/>
-      <c r="D14" s="23"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="5"/>
-      <c r="F14" s="21"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="21"/>
+      <c r="H14" s="15"/>
       <c r="I14" s="5"/>
       <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="16"/>
+      <c r="A15" s="21"/>
       <c r="C15" s="5"/>
-      <c r="D15" s="23"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="5"/>
-      <c r="F15" s="21"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="21"/>
+      <c r="H15" s="15"/>
       <c r="I15" s="5"/>
       <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="16"/>
+      <c r="A16" s="21"/>
       <c r="C16" s="5"/>
-      <c r="D16" s="23"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="5"/>
-      <c r="F16" s="21"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="6"/>
-      <c r="H16" s="21"/>
+      <c r="H16" s="15"/>
       <c r="I16" s="7"/>
       <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="16"/>
+      <c r="A17" s="21"/>
       <c r="C17" s="5"/>
-      <c r="D17" s="23"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="5"/>
-      <c r="F17" s="21"/>
+      <c r="F17" s="15"/>
       <c r="G17" s="6"/>
-      <c r="H17" s="21"/>
+      <c r="H17" s="15"/>
       <c r="I17" s="7"/>
       <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="17"/>
+      <c r="A18" s="23"/>
       <c r="C18" s="5"/>
-      <c r="D18" s="24"/>
+      <c r="D18" s="19"/>
       <c r="E18" s="5"/>
-      <c r="F18" s="22"/>
+      <c r="F18" s="16"/>
       <c r="G18" s="6"/>
-      <c r="H18" s="21"/>
+      <c r="H18" s="15"/>
       <c r="I18" s="7"/>
       <c r="K18" s="5"/>
     </row>
@@ -2442,30 +2182,20 @@
       <c r="K19" s="5"/>
     </row>
     <row r="21" spans="1:11" ht="28.5">
-      <c r="A21" s="15" t="s">
-        <v>6</v>
+      <c r="A21" s="20" t="s">
+        <v>1</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="C21" s="1"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="E21" s="1"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="G21" s="3"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="I21" s="3"/>
+      <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="16"/>
+      <c r="A22" s="21"/>
       <c r="C22" s="5"/>
       <c r="E22" s="5"/>
       <c r="G22" s="5"/>
@@ -2473,7 +2203,7 @@
       <c r="K22" s="5"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="20"/>
+      <c r="A23" s="22"/>
       <c r="C23" s="5"/>
       <c r="E23" s="5"/>
       <c r="G23" s="5"/>
@@ -2481,7 +2211,7 @@
       <c r="K23" s="5"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="20"/>
+      <c r="A24" s="22"/>
       <c r="C24" s="5"/>
       <c r="E24" s="5"/>
       <c r="G24" s="5"/>
@@ -2489,7 +2219,7 @@
       <c r="K24" s="5"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="20"/>
+      <c r="A25" s="22"/>
       <c r="C25" s="5"/>
       <c r="E25" s="5"/>
       <c r="G25" s="5"/>
@@ -2497,7 +2227,7 @@
       <c r="K25" s="5"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="20"/>
+      <c r="A26" s="22"/>
       <c r="C26" s="5"/>
       <c r="E26" s="5"/>
       <c r="G26" s="5"/>
@@ -2505,7 +2235,7 @@
       <c r="K26" s="5"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="20"/>
+      <c r="A27" s="22"/>
       <c r="C27" s="5"/>
       <c r="E27" s="5"/>
       <c r="G27" s="5"/>
@@ -2513,7 +2243,7 @@
       <c r="K27" s="5"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="20"/>
+      <c r="A28" s="22"/>
       <c r="C28" s="5"/>
       <c r="E28" s="5"/>
       <c r="G28" s="5"/>
@@ -2521,7 +2251,7 @@
       <c r="K28" s="5"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="16"/>
+      <c r="A29" s="21"/>
       <c r="C29" s="5"/>
       <c r="E29" s="5"/>
       <c r="G29" s="5"/>
@@ -2529,7 +2259,7 @@
       <c r="K29" s="5"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="16"/>
+      <c r="A30" s="21"/>
       <c r="C30" s="5"/>
       <c r="E30" s="5"/>
       <c r="G30" s="5"/>
@@ -2537,7 +2267,7 @@
       <c r="K30" s="5"/>
     </row>
     <row r="31" spans="1:11">
-      <c r="A31" s="16"/>
+      <c r="A31" s="21"/>
       <c r="C31" s="5"/>
       <c r="E31" s="5"/>
       <c r="G31" s="5"/>
@@ -2545,7 +2275,7 @@
       <c r="K31" s="5"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="16"/>
+      <c r="A32" s="21"/>
       <c r="C32" s="5"/>
       <c r="E32" s="5"/>
       <c r="G32" s="5"/>
@@ -2553,7 +2283,7 @@
       <c r="K32" s="5"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="16"/>
+      <c r="A33" s="21"/>
       <c r="C33" s="5"/>
       <c r="E33" s="5"/>
       <c r="G33" s="5"/>
@@ -2561,7 +2291,7 @@
       <c r="K33" s="5"/>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="16"/>
+      <c r="A34" s="21"/>
       <c r="C34" s="7"/>
       <c r="E34" s="5"/>
       <c r="G34" s="5"/>
@@ -2569,7 +2299,7 @@
       <c r="K34" s="7"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="17"/>
+      <c r="A35" s="23"/>
       <c r="C35" s="7"/>
       <c r="E35" s="5"/>
       <c r="G35" s="5"/>
@@ -2585,30 +2315,20 @@
       <c r="K36" s="5"/>
     </row>
     <row r="38" spans="1:11" ht="28.5">
-      <c r="A38" s="15" t="s">
-        <v>12</v>
+      <c r="A38" s="20" t="s">
+        <v>2</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="C38" s="1"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="E38" s="1"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="G38" s="3"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K38" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="I38" s="3"/>
+      <c r="K38" s="1"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="16"/>
+      <c r="A39" s="21"/>
       <c r="C39" s="5"/>
       <c r="D39" s="11"/>
       <c r="E39" s="5"/>
@@ -2617,7 +2337,7 @@
       <c r="K39" s="5"/>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="16"/>
+      <c r="A40" s="21"/>
       <c r="C40" s="5"/>
       <c r="D40" s="12"/>
       <c r="E40" s="5"/>
@@ -2626,7 +2346,7 @@
       <c r="K40" s="5"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="16"/>
+      <c r="A41" s="21"/>
       <c r="C41" s="5"/>
       <c r="D41" s="12"/>
       <c r="E41" s="5"/>
@@ -2635,7 +2355,7 @@
       <c r="K41" s="5"/>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="16"/>
+      <c r="A42" s="21"/>
       <c r="C42" s="5"/>
       <c r="D42" s="12"/>
       <c r="E42" s="5"/>
@@ -2644,7 +2364,7 @@
       <c r="K42" s="7"/>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="20"/>
+      <c r="A43" s="22"/>
       <c r="C43" s="5"/>
       <c r="D43" s="12"/>
       <c r="E43" s="5"/>
@@ -2653,7 +2373,7 @@
       <c r="K43" s="7"/>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="20"/>
+      <c r="A44" s="22"/>
       <c r="C44" s="5"/>
       <c r="D44" s="12"/>
       <c r="E44" s="5"/>
@@ -2662,7 +2382,7 @@
       <c r="K44" s="7"/>
     </row>
     <row r="45" spans="1:11">
-      <c r="A45" s="20"/>
+      <c r="A45" s="22"/>
       <c r="C45" s="5"/>
       <c r="D45" s="12"/>
       <c r="E45" s="5"/>
@@ -2671,7 +2391,7 @@
       <c r="K45" s="7"/>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="20"/>
+      <c r="A46" s="22"/>
       <c r="C46" s="5"/>
       <c r="D46" s="12"/>
       <c r="E46" s="5"/>
@@ -2680,7 +2400,7 @@
       <c r="K46" s="7"/>
     </row>
     <row r="47" spans="1:11">
-      <c r="A47" s="20"/>
+      <c r="A47" s="22"/>
       <c r="C47" s="5"/>
       <c r="D47" s="12"/>
       <c r="E47" s="5"/>
@@ -2689,7 +2409,7 @@
       <c r="K47" s="7"/>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="20"/>
+      <c r="A48" s="22"/>
       <c r="C48" s="5"/>
       <c r="D48" s="12"/>
       <c r="E48" s="5"/>
@@ -2698,7 +2418,7 @@
       <c r="K48" s="7"/>
     </row>
     <row r="49" spans="1:11">
-      <c r="A49" s="20"/>
+      <c r="A49" s="22"/>
       <c r="C49" s="5"/>
       <c r="D49" s="12"/>
       <c r="E49" s="5"/>
@@ -2707,7 +2427,7 @@
       <c r="K49" s="7"/>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="20"/>
+      <c r="A50" s="22"/>
       <c r="C50" s="5"/>
       <c r="D50" s="12"/>
       <c r="E50" s="5"/>
@@ -2716,7 +2436,7 @@
       <c r="K50" s="7"/>
     </row>
     <row r="51" spans="1:11">
-      <c r="A51" s="16"/>
+      <c r="A51" s="21"/>
       <c r="C51" s="5"/>
       <c r="D51" s="12"/>
       <c r="E51" s="5"/>
@@ -2725,7 +2445,7 @@
       <c r="K51" s="7"/>
     </row>
     <row r="52" spans="1:11">
-      <c r="A52" s="16"/>
+      <c r="A52" s="21"/>
       <c r="C52" s="5"/>
       <c r="D52" s="12"/>
       <c r="E52" s="5"/>
@@ -2734,7 +2454,7 @@
       <c r="K52" s="7"/>
     </row>
     <row r="53" spans="1:11">
-      <c r="A53" s="17"/>
+      <c r="A53" s="23"/>
       <c r="C53" s="5"/>
       <c r="D53" s="12"/>
       <c r="E53" s="5"/>
@@ -2743,30 +2463,20 @@
       <c r="K53" s="7"/>
     </row>
     <row r="55" spans="1:11" ht="28.5">
-      <c r="A55" s="15" t="s">
-        <v>18</v>
+      <c r="A55" s="20" t="s">
+        <v>3</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="C55" s="1"/>
       <c r="D55" s="2"/>
-      <c r="E55" s="1" t="s">
-        <v>20</v>
-      </c>
+      <c r="E55" s="1"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="G55" s="3"/>
       <c r="H55" s="2"/>
-      <c r="I55" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="I55" s="3"/>
+      <c r="K55" s="1"/>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="16"/>
+      <c r="A56" s="21"/>
       <c r="C56" s="5"/>
       <c r="E56" s="5"/>
       <c r="G56" s="5"/>
@@ -2774,7 +2484,7 @@
       <c r="K56" s="5"/>
     </row>
     <row r="57" spans="1:11">
-      <c r="A57" s="16"/>
+      <c r="A57" s="21"/>
       <c r="C57" s="5"/>
       <c r="E57" s="5"/>
       <c r="G57" s="5"/>
@@ -2782,7 +2492,7 @@
       <c r="K57" s="5"/>
     </row>
     <row r="58" spans="1:11">
-      <c r="A58" s="16"/>
+      <c r="A58" s="21"/>
       <c r="C58" s="5"/>
       <c r="E58" s="5"/>
       <c r="G58" s="5"/>
@@ -2790,7 +2500,7 @@
       <c r="K58" s="5"/>
     </row>
     <row r="59" spans="1:11">
-      <c r="A59" s="16"/>
+      <c r="A59" s="21"/>
       <c r="C59" s="5"/>
       <c r="E59" s="5"/>
       <c r="G59" s="5"/>
@@ -2798,7 +2508,7 @@
       <c r="K59" s="5"/>
     </row>
     <row r="60" spans="1:11">
-      <c r="A60" s="20"/>
+      <c r="A60" s="22"/>
       <c r="C60" s="5"/>
       <c r="E60" s="5"/>
       <c r="G60" s="5"/>
@@ -2806,7 +2516,7 @@
       <c r="K60" s="5"/>
     </row>
     <row r="61" spans="1:11">
-      <c r="A61" s="20"/>
+      <c r="A61" s="22"/>
       <c r="C61" s="5"/>
       <c r="E61" s="5"/>
       <c r="G61" s="5"/>
@@ -2814,7 +2524,7 @@
       <c r="K61" s="5"/>
     </row>
     <row r="62" spans="1:11">
-      <c r="A62" s="20"/>
+      <c r="A62" s="22"/>
       <c r="C62" s="5"/>
       <c r="E62" s="5"/>
       <c r="G62" s="5"/>
@@ -2822,7 +2532,7 @@
       <c r="K62" s="5"/>
     </row>
     <row r="63" spans="1:11">
-      <c r="A63" s="20"/>
+      <c r="A63" s="22"/>
       <c r="C63" s="5"/>
       <c r="E63" s="5"/>
       <c r="G63" s="5"/>
@@ -2830,7 +2540,7 @@
       <c r="K63" s="5"/>
     </row>
     <row r="64" spans="1:11">
-      <c r="A64" s="20"/>
+      <c r="A64" s="22"/>
       <c r="C64" s="5"/>
       <c r="E64" s="5"/>
       <c r="G64" s="5"/>
@@ -2838,7 +2548,7 @@
       <c r="K64" s="5"/>
     </row>
     <row r="65" spans="1:11">
-      <c r="A65" s="20"/>
+      <c r="A65" s="22"/>
       <c r="C65" s="5"/>
       <c r="E65" s="5"/>
       <c r="G65" s="5"/>
@@ -2846,7 +2556,7 @@
       <c r="K65" s="5"/>
     </row>
     <row r="66" spans="1:11">
-      <c r="A66" s="16"/>
+      <c r="A66" s="21"/>
       <c r="C66" s="5"/>
       <c r="E66" s="5"/>
       <c r="G66" s="5"/>
@@ -2854,7 +2564,7 @@
       <c r="K66" s="5"/>
     </row>
     <row r="67" spans="1:11">
-      <c r="A67" s="16"/>
+      <c r="A67" s="21"/>
       <c r="C67" s="7"/>
       <c r="E67" s="5"/>
       <c r="G67" s="5"/>
@@ -2862,7 +2572,7 @@
       <c r="K67" s="5"/>
     </row>
     <row r="68" spans="1:11">
-      <c r="A68" s="16"/>
+      <c r="A68" s="21"/>
       <c r="C68" s="7"/>
       <c r="E68" s="5"/>
       <c r="G68" s="5"/>
@@ -2870,7 +2580,7 @@
       <c r="K68" s="5"/>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="16"/>
+      <c r="A69" s="21"/>
       <c r="C69" s="7"/>
       <c r="E69" s="5"/>
       <c r="G69" s="5"/>
@@ -2878,7 +2588,7 @@
       <c r="K69" s="5"/>
     </row>
     <row r="70" spans="1:11">
-      <c r="A70" s="17"/>
+      <c r="A70" s="23"/>
       <c r="C70" s="7"/>
       <c r="E70" s="5"/>
       <c r="G70" s="7"/>
@@ -2886,93 +2596,89 @@
       <c r="K70" s="5"/>
     </row>
     <row r="72" spans="1:11" ht="28.5">
-      <c r="A72" s="15" t="s">
-        <v>24</v>
+      <c r="A72" s="20" t="s">
+        <v>4</v>
       </c>
-      <c r="C72" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="C72" s="1"/>
+      <c r="E72" s="3"/>
     </row>
     <row r="73" spans="1:11">
-      <c r="A73" s="16"/>
+      <c r="A73" s="21"/>
       <c r="C73" s="4"/>
-      <c r="E73" s="14"/>
+      <c r="E73" s="13"/>
     </row>
     <row r="74" spans="1:11">
-      <c r="A74" s="16"/>
+      <c r="A74" s="21"/>
       <c r="C74" s="5"/>
       <c r="E74" s="5"/>
     </row>
     <row r="75" spans="1:11">
-      <c r="A75" s="16"/>
+      <c r="A75" s="21"/>
       <c r="C75" s="5"/>
       <c r="E75" s="5"/>
     </row>
     <row r="76" spans="1:11">
-      <c r="A76" s="20"/>
+      <c r="A76" s="22"/>
       <c r="C76" s="5"/>
       <c r="E76" s="5"/>
     </row>
     <row r="77" spans="1:11">
-      <c r="A77" s="20"/>
+      <c r="A77" s="22"/>
       <c r="C77" s="5"/>
       <c r="E77" s="5"/>
     </row>
     <row r="78" spans="1:11">
-      <c r="A78" s="20"/>
+      <c r="A78" s="22"/>
       <c r="C78" s="5"/>
       <c r="E78" s="5"/>
     </row>
     <row r="79" spans="1:11">
-      <c r="A79" s="20"/>
+      <c r="A79" s="22"/>
       <c r="C79" s="5"/>
       <c r="E79" s="5"/>
     </row>
     <row r="80" spans="1:11">
-      <c r="A80" s="20"/>
+      <c r="A80" s="22"/>
       <c r="C80" s="5"/>
       <c r="E80" s="5"/>
     </row>
     <row r="81" spans="1:5">
-      <c r="A81" s="20"/>
+      <c r="A81" s="22"/>
       <c r="C81" s="5"/>
       <c r="E81" s="5"/>
     </row>
     <row r="82" spans="1:5">
-      <c r="A82" s="20"/>
+      <c r="A82" s="22"/>
       <c r="C82" s="5"/>
       <c r="E82" s="5"/>
     </row>
     <row r="83" spans="1:5">
-      <c r="A83" s="20"/>
+      <c r="A83" s="22"/>
       <c r="C83" s="5"/>
       <c r="E83" s="5"/>
     </row>
     <row r="84" spans="1:5">
-      <c r="A84" s="16"/>
+      <c r="A84" s="21"/>
       <c r="C84" s="5"/>
       <c r="E84" s="5"/>
     </row>
     <row r="85" spans="1:5">
-      <c r="A85" s="20"/>
+      <c r="A85" s="22"/>
       <c r="C85" s="5"/>
       <c r="E85" s="5"/>
     </row>
     <row r="86" spans="1:5">
-      <c r="A86" s="20"/>
+      <c r="A86" s="22"/>
       <c r="C86" s="5"/>
       <c r="E86" s="5"/>
     </row>
     <row r="87" spans="1:5">
-      <c r="A87" s="16"/>
+      <c r="A87" s="21"/>
       <c r="C87" s="5"/>
       <c r="E87" s="5"/>
     </row>
     <row r="88" spans="1:5">
-      <c r="A88" s="17"/>
+      <c r="A88" s="23"/>
       <c r="C88" s="5"/>
       <c r="E88" s="5"/>
     </row>

</xml_diff>